<commit_message>
Update features spreadsheet with new data
</commit_message>
<xml_diff>
--- a/docs/fuatures.xlsx
+++ b/docs/fuatures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\L67\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04DFCAE9-D0A0-4675-9EA5-825B5550B25F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DFCE46-77B9-4F67-82A9-8D36FF81D148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{27C0ACFE-F6C5-4C78-8331-F8ADD4815FE8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="135">
   <si>
     <t>MARKA</t>
   </si>
@@ -186,6 +186,261 @@
   </si>
   <si>
     <t>45 KM</t>
+  </si>
+  <si>
+    <t>5,4 KW</t>
+  </si>
+  <si>
+    <t>6 KW</t>
+  </si>
+  <si>
+    <t>JANT</t>
+  </si>
+  <si>
+    <t>ŞARJ 1</t>
+  </si>
+  <si>
+    <t>4 SAAT</t>
+  </si>
+  <si>
+    <t>PİL</t>
+  </si>
+  <si>
+    <t>LİTYUM-İYON</t>
+  </si>
+  <si>
+    <t>MAX AĞIR.</t>
+  </si>
+  <si>
+    <t>BOŞ AĞIR.</t>
+  </si>
+  <si>
+    <t>TOPOLINO PLUS</t>
+  </si>
+  <si>
+    <t>ÖN FREN</t>
+  </si>
+  <si>
+    <t>ARKA FREN</t>
+  </si>
+  <si>
+    <t>DİSK</t>
+  </si>
+  <si>
+    <t>KAMPANA</t>
+  </si>
+  <si>
+    <t>60 KM</t>
+  </si>
+  <si>
+    <t>155/65 R14</t>
+  </si>
+  <si>
+    <t>125/65 R12</t>
+  </si>
+  <si>
+    <t>340 KG</t>
+  </si>
+  <si>
+    <t>483 KG</t>
+  </si>
+  <si>
+    <t>470 KG</t>
+  </si>
+  <si>
+    <t>487 KG</t>
+  </si>
+  <si>
+    <t>700 KG</t>
+  </si>
+  <si>
+    <t>600 KG</t>
+  </si>
+  <si>
+    <t>8 SAAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAPASİTE </t>
+  </si>
+  <si>
+    <t>4 KİŞİ</t>
+  </si>
+  <si>
+    <t>145/70 R12</t>
+  </si>
+  <si>
+    <t>424 KG</t>
+  </si>
+  <si>
+    <t>687 KG</t>
+  </si>
+  <si>
+    <t>2 KİŞİ</t>
+  </si>
+  <si>
+    <t>3 KİŞİ</t>
+  </si>
+  <si>
+    <t>80 KM</t>
+  </si>
+  <si>
+    <t>6 SAAT</t>
+  </si>
+  <si>
+    <t>448 KG</t>
+  </si>
+  <si>
+    <t>897 KG</t>
+  </si>
+  <si>
+    <t>KLİMA</t>
+  </si>
+  <si>
+    <t>72V146 Ah Lithium</t>
+  </si>
+  <si>
+    <t>120 KM</t>
+  </si>
+  <si>
+    <t>UZUNLUK</t>
+  </si>
+  <si>
+    <t>GENİŞLİK</t>
+  </si>
+  <si>
+    <t>YÜKSEKLİK</t>
+  </si>
+  <si>
+    <t>2245 mm</t>
+  </si>
+  <si>
+    <t>1290 mm</t>
+  </si>
+  <si>
+    <t>1570 mm</t>
+  </si>
+  <si>
+    <t>72V58AH</t>
+  </si>
+  <si>
+    <t>72V58AH JEL</t>
+  </si>
+  <si>
+    <t>72V100AH</t>
+  </si>
+  <si>
+    <t>DİNGİL</t>
+  </si>
+  <si>
+    <t>VAR</t>
+  </si>
+  <si>
+    <t>1650 mm</t>
+  </si>
+  <si>
+    <t>2605 mm</t>
+  </si>
+  <si>
+    <t>1295 mm</t>
+  </si>
+  <si>
+    <t>1610 mm</t>
+  </si>
+  <si>
+    <t>2670 mm</t>
+  </si>
+  <si>
+    <t>1400 mm</t>
+  </si>
+  <si>
+    <t>1625 mm</t>
+  </si>
+  <si>
+    <t>1665 mm</t>
+  </si>
+  <si>
+    <t>1500 mm</t>
+  </si>
+  <si>
+    <t>2535 mm</t>
+  </si>
+  <si>
+    <t>1530 mm</t>
+  </si>
+  <si>
+    <t>1730 mm</t>
+  </si>
+  <si>
+    <t>2460 mm</t>
+  </si>
+  <si>
+    <t>1390 mm</t>
+  </si>
+  <si>
+    <t>1525 mm</t>
+  </si>
+  <si>
+    <t>1728 mm</t>
+  </si>
+  <si>
+    <t>ISITMA</t>
+  </si>
+  <si>
+    <t>TOPOLINO DOLCEVİTA</t>
+  </si>
+  <si>
+    <t>2,5 KW</t>
+  </si>
+  <si>
+    <t>3KİŞİ</t>
+  </si>
+  <si>
+    <t>1215 mm</t>
+  </si>
+  <si>
+    <t>1680 mm</t>
+  </si>
+  <si>
+    <t>1635 mm</t>
+  </si>
+  <si>
+    <t>400 KG</t>
+  </si>
+  <si>
+    <t>135/70 R12</t>
+  </si>
+  <si>
+    <t>90 KM</t>
+  </si>
+  <si>
+    <t>640 KG</t>
+  </si>
+  <si>
+    <t>228 KM</t>
+  </si>
+  <si>
+    <t>496 KM</t>
+  </si>
+  <si>
+    <t>200 KM</t>
+  </si>
+  <si>
+    <t>12,4 KW</t>
+  </si>
+  <si>
+    <t>145/70 R13</t>
+  </si>
+  <si>
+    <t>2519 mm</t>
+  </si>
+  <si>
+    <t>1473 mm</t>
+  </si>
+  <si>
+    <t>1501 mm</t>
+  </si>
+  <si>
+    <t>1566 mm</t>
   </si>
 </sst>
 </file>
@@ -195,13 +450,27 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;₺&quot;#,##0"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -225,11 +494,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -565,17 +843,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA656D03-4022-47D2-ACAD-D521290195B3}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
     <col min="2" max="2" width="21.42578125" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="1"/>
+    <col min="3" max="3" width="10.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" style="2" customWidth="1"/>
-    <col min="5" max="6" width="9.140625" style="2"/>
+    <col min="5" max="5" width="20.85546875" style="3" customWidth="1"/>
+    <col min="6" max="7" width="9.140625" style="2"/>
+    <col min="8" max="8" width="15.7109375" customWidth="1"/>
+    <col min="10" max="10" width="13" style="2" customWidth="1"/>
+    <col min="11" max="11" width="10.85546875" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" customWidth="1"/>
+    <col min="13" max="13" width="11.28515625" customWidth="1"/>
+    <col min="14" max="14" width="9.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.140625" style="2"/>
+    <col min="17" max="17" width="11" customWidth="1"/>
+    <col min="18" max="18" width="12.28515625" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" customWidth="1"/>
+    <col min="20" max="20" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -588,14 +878,56 @@
       <c r="D1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -608,14 +940,54 @@
       <c r="D2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>48</v>
+      <c r="E2" s="4" t="s">
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>5</v>
       </c>
@@ -625,14 +997,50 @@
       <c r="D3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>48</v>
+      <c r="E3" s="3" t="s">
+        <v>95</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -642,14 +1050,54 @@
       <c r="D4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H4" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -659,181 +1107,639 @@
       <c r="C5" s="1">
         <v>585000</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="S5" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1">
+        <v>595000</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C7" s="1">
         <v>605000</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="1">
-        <v>595000</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="C8" s="1">
+        <v>669900</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="1">
+        <v>714900</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="R9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" s="1">
+        <v>575900</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="R10" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="S10" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B11" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="C11" s="1">
+        <v>299520</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="S11" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="C12" s="1">
+        <v>279900</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="S12" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>16</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B13" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+      <c r="C13" s="1">
+        <v>1652440</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="C14" s="1">
+        <v>1274510</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>18</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B15" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>20</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B16" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>25</v>
+      </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>30</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B23" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>32</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B24" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>36</v>
-      </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>40</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B31" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update source URLs and modify features spreadsheet
</commit_message>
<xml_diff>
--- a/docs/fuatures.xlsx
+++ b/docs/fuatures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\L67\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DFCE46-77B9-4F67-82A9-8D36FF81D148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E8A309-E089-4CC4-8D4D-F6D253BDCC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{27C0ACFE-F6C5-4C78-8331-F8ADD4815FE8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="154">
   <si>
     <t>MARKA</t>
   </si>
@@ -419,9 +419,6 @@
     <t>228 KM</t>
   </si>
   <si>
-    <t>496 KM</t>
-  </si>
-  <si>
     <t>200 KM</t>
   </si>
   <si>
@@ -441,6 +438,66 @@
   </si>
   <si>
     <t>1566 mm</t>
+  </si>
+  <si>
+    <t>76,8V100AH</t>
+  </si>
+  <si>
+    <t>70 KM</t>
+  </si>
+  <si>
+    <t>TAMBUR</t>
+  </si>
+  <si>
+    <t>2850 mm</t>
+  </si>
+  <si>
+    <t>1540 mm</t>
+  </si>
+  <si>
+    <t>1940 mm</t>
+  </si>
+  <si>
+    <t>15 KW</t>
+  </si>
+  <si>
+    <t>215 KM</t>
+  </si>
+  <si>
+    <t>2/4 KİŞİ</t>
+  </si>
+  <si>
+    <t>496 KG</t>
+  </si>
+  <si>
+    <t>449 KG</t>
+  </si>
+  <si>
+    <t>5 SAAT</t>
+  </si>
+  <si>
+    <t>100 KM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7,5 KW </t>
+  </si>
+  <si>
+    <t>LiFePO4</t>
+  </si>
+  <si>
+    <t>KAREA</t>
+  </si>
+  <si>
+    <t>FIT</t>
+  </si>
+  <si>
+    <t>LFP</t>
+  </si>
+  <si>
+    <t>135 KM</t>
+  </si>
+  <si>
+    <t>12 KW</t>
   </si>
 </sst>
 </file>
@@ -843,7 +900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA656D03-4022-47D2-ACAD-D521290195B3}">
-  <dimension ref="A1:T31"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -1439,69 +1496,62 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" t="s">
+        <v>150</v>
+      </c>
+      <c r="C11" s="1">
+        <v>699000</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2">
+        <v>540</v>
+      </c>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2">
+        <v>2631</v>
+      </c>
+      <c r="R11" s="2">
+        <v>1498</v>
+      </c>
+      <c r="S11" s="2">
+        <v>1621</v>
+      </c>
+      <c r="T11" s="2"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C12" s="1">
         <v>299520</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="P11" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="Q11" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="R11" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="S11" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="T11" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="1">
-        <v>279900</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>117</v>
@@ -1553,193 +1603,387 @@
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="1">
+        <v>279900</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="S13" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>16</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C14" s="1">
         <v>1652440</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="R13" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="1">
-        <v>1274510</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>130</v>
-      </c>
       <c r="J14" s="2" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="N14" s="2" t="s">
         <v>79</v>
       </c>
+      <c r="O14" s="2" t="s">
+        <v>98</v>
+      </c>
       <c r="Q14" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="R14" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="R14" s="2" t="s">
+      <c r="S14" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="S14" s="2" t="s">
+      <c r="T14" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="T14" s="2" t="s">
-        <v>134</v>
-      </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>18</v>
-      </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="C15" s="1">
+        <v>1274510</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="1">
+        <v>650000</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>20</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="C17" s="1">
+        <v>765000</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q17">
+        <v>3060</v>
+      </c>
+      <c r="R17">
+        <v>1500</v>
+      </c>
+      <c r="S17">
+        <v>1620</v>
+      </c>
+      <c r="T17">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>22</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
+      <c r="C18" s="1">
+        <v>489000</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J18" s="2">
+        <v>471</v>
+      </c>
+      <c r="K18" s="2">
+        <v>700</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q18">
+        <v>2494</v>
+      </c>
+      <c r="R18">
+        <v>1649</v>
+      </c>
+      <c r="S18">
+        <v>1334</v>
+      </c>
+      <c r="T18">
+        <v>1668</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="C19" s="1">
+        <v>399000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>25</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>30</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>32</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>36</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>40</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>